<commit_message>
feat(candyshots): confirmar regimen general (IVA recuperable) y guardar el generador
- INICIO!C6 = SI: Fabian confirma RUC en regimen general con credito tributario
- Costos bajan ~13%: el IVA de insumos deja de ser costo
- Margen granizado maquina 78.4% · equilibrio 20 vasos/dia
- scripts/generar-sheet-candyshots.py: generador reproducible del .xlsx
- finanzas/analisis-costos.md marcado como superado por el Sheets

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/abrir-candyshots/administracion/CandyShots-Administracion.xlsx
+++ b/projects/abrir-candyshots/administracion/CandyShots-Administracion.xlsx
@@ -854,12 +854,12 @@
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>SI = tienes RUC régimen general y haces crédito tributario. NO = RIMPE/no facturas, el IVA es costo.</t>
+          <t>CONFIRMADO 2026-09-07: SI. Regimen general con RUC, credito tributario. Si eso cambia, ponlo en NO.</t>
         </is>
       </c>
     </row>

</xml_diff>